<commit_message>
Feedback workbook rows 5-6: wireframe-comparison self-catches
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -643,6 +643,86 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Home — hero change line</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>(self-caught while re-reading the approved wireframe at founder request)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Approved wireframe says "up $11,200 this month ▲up" — DOLLARS, with percent. The build showed percent only.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Change line now shows dollars AND percent ("▲ up $11,200 (1.4%) this month"), both derived from the same measured return via one helper (periodDollarDelta) so they can never disagree. Pinned with the wireframe's own numbers.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>mockups/approved-wireframes-home-networth-dd-v1.1.html</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Home — investments info dot (re-classified)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>(re-classification of row 2 after checking the approved design)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>The investments info dot was row c1 of the APPROVED detailed design all along ("stocks &amp; funds + bonds + alternatives — cash is counted separately") — row 2 was a missed approved-design row, not a new request. The 2026-07-18 comment audit marked info dots closed after adding only the net-worth and market dots.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Glossary text now uses the approved c1 wording plus the investments-vs-net-worth distinction asked for in row 2.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>mockups/approved-wireframes-home-networth-dd-v1.1.html</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Standing order: full-color hi-fi mockups only + first two delivered (Home, Net worth — Build 44 preview)
Both states drawn (rich + first-day) with the app's real theme tokens.
CLAUDE.md MOCK-FIRST updated; workbook row 7.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -723,6 +723,46 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Process — mock fidelity</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Going forward — I want full colored high fidelity mockups.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>The audit-round mocks were hi-fi HTML but the folder-saved wireframes were ASCII transcriptions.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>ADOPTED as a standing rule (CLAUDE.md MOCK-FIRST): every mock is a full-color hi-fi HTML phone frame using the app's real theme tokens, showing BOTH rich and empty/first-day states. First two delivered for Build 44 approval: home-v2-hifi + networth-v2-hifi.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>mockups/home-v2-hifi-2026-07-19.html · mockups/networth-v2-hifi-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>ADOPTED — mocks awaiting your approval</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Net worth mock v3+v4: account rows under each asset type; v4 adds INTERACTIVE expand/collapse (awaiting founder approval before code change)
v2's missing nested accounts + non-summing totals fixed; v4 is tappable in
the browser. Workbook row 8.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -763,6 +763,46 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Net worth — accounts under asset types</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>We agreed to add account-level details under the asset type — not reflected in the mockup. In expandable and collapse form.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>The BUILT screen already lists accounts under each class (NetWorthScreen.tsx:408, always visible, 5-cap + "all N"). The v2 mock failed to draw them, and its class totals did not sum to the OWN total. The expand/collapse behavior is NEW direction (today): built screen shows them always-visible.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Mock v4 drawn INTERACTIVE (click class rows to expand/collapse; default collapsed; caret word+motion, never color alone; single class auto-expands on first day; 5-cap kept). CODE CHANGE AWAITS YOUR APPROVAL of v4 — then the screen gets per-class expand/collapse to match.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>mockups/networth-v4-hifi-expandable-2026-07-19.html (v3 kept as iteration record)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>MOCK READY — awaiting approval</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Build-43 device findings R2: v4 expand/collapse BUILT (approved) + label dedupe/mask + cursor self-heal + MMF=cash + readable CUSIP names; v5 class-split mock awaits approval
Finding 1: accountDisplayName — institution never doubles, broker mask tells
twins apart (pinned with the founder's exact E*TRADE case).
Finding 2: money-market tickers class as CASH (engine, pinned); the full
per-class SPLIT of mixed accounts is mocked (networth-v5) for approval.
Finding 3: envelope fix was already in; NEW self-heal — a cursor with no
ledger rows behind it is ignored, full history refetches (Build 43 advanced
cursors over zero rows; devices repair themselves on Build 44's first sync).
Finding 4: CUSIP-style tickers display the security's readable name.
v4 expand/collapse: default collapsed, caret + word, lone class auto-expands;
W8 walk updated to the new interaction. 1235 green. Workbook rows 9-12.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -803,6 +803,166 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Net worth — duplicate account labels</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Two imported E*TRADE accounts both labelled "E-Trade E*Trade Individua…".</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>The row prefixed the institution onto a label that already contains the institution ("E-Trade" + "E*Trade Individual Brokerage"), and the broker's account mask was never shown — so the twins were identical.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>One canonical accountDisplayName helper: institution prefixes ONLY when the label doesn't already say it; the broker mask (••9Cmw / ••D9LA) suffixes so twins are tellable apart. Pinned with your exact case.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>n/a (matches approved wireframe "Brokerage ...4821")</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Net worth — mixed account all under Stocks/ETFs</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Both accounts listed under Stocks/ETFs. Total accurate, but not separating CD from options from stock/ETF from cash in the account.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>The class table books an account's WHOLE balance to one class; a connected brokerage with positions lands entirely under Stocks/ETFs even when it holds CDs, money market, cash and options. Also: E*TRADE doesn't flag money-market funds, so VMFXX classed as stocks.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>TWO parts: (a) engine truth DONE — money-market tickers (VMFXX etc.) now class as cash, pinned; (b) the class SPLIT (account appears under each class it holds, portions sum exactly to the broker total) is drawn in mock v5 — AWAITING YOUR APPROVAL before building.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>mockups/networth-v5-hifi-class-split-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>PART FIXED · v5 MOCK AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Transactions — no activity imported</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>No activity imported.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>KNOWN + FIXED after Build 43 was cut: SnapTrade wraps history in a pagination envelope the docs never showed; Build 43's guard silently dropped it (found same day in the live relay test with a real account). WORSE: Build 43 still advanced the sync cursor, so without repair Build 44 would fetch only the last week and orphan your history.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Envelope fix was already in (pinned with the live shape). NEW self-heal added today: a cursor with no ledger rows behind it is ignored and the FULL history refetches — your device repairs itself automatically on Build 44's first sync. Both pinned.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>n/a (engine)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — history arrives on Build 44's first sync</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Account detail — is this what you built?</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>E-Trade E*Trade Individual Brokerage → $, Stocks/ETFs Taxable, holds 49306sx43. lctx. vmfxx, OPTIONS IN THIS ACCOUNT QQQ $600 put… counted inside this account's total. Is this what you built?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>YES — that is the built screen (balance + class/wrapper line + holdings line + itemized options with the counted-inside note). Three parts of it were wrong, though: the doubled name (row 9), the "Stocks/ETFs" class line for a mixed account (row 10), and "49306SX43" — a raw CUSIP identifier where a human-readable name belongs.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>CUSIP-style tickers now display the security's NAME (e.g. "CD 4.30% due 2027…" instead of 49306SX43); name captured at sync. The class-line follows row 10's v5 decision.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>FIXED (names) · class line follows v5</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
R3: scrambled broker ids never shown as masks (digit-only + stable ordinals) + FULL-SCREEN mock rule; v6 + account-detail mocks delivered
Founder catch: '9Cmw/D9LA' are E*TRADE's scrambled ids, not account digits.
Masks now require 4 real digits; identical twins get ' · 1 / · 2' (stable
order); detail header uses the same name. Pinned both ways (display + ingest).
Mocks: networth-v6 full screen (hero→tab bar, split carried in, sums exact)
supersedes v5 as the approval target; account-detail-v1 shows the tap-through
page. CLAUDE.md: mocks are always the full screen and their numbers add up.
1236 green. Workbook rows 13-14.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -963,6 +963,86 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Net worth — "9Cmw / D9LA" masks</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>What is 9Cmw and D9LA — these are not the last 4 digits of the account.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Correct. E*TRADE refuses to share the real account number; SnapTrade relays a SCRAMBLED identifier instead, and the code blindly took its last 4 characters. Gibberish shown as if it were your account digits.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>A mask now exists ONLY when the tail is 4 real digits (brokers that share them show "••4821"). Otherwise identical twins get a stable "· 1 / · 2" ordinal (ordered so numbering never shuffles); accounts stay renamable on their page. Pinned with both cases.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>shown in v6 mock</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Process — mock completeness + account-detail mock</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Why is the mockup missing the hero and rest of the screen? Also create a mockup of the screen when I click on a particular account.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>The v5 mock cropped to the one card under discussion — against the spirit of the hi-fi order.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Standing rule added: mocks show the FULL screen top to bottom, and their numbers must add up. Delivered: networth-v6 FULL-SCREEN mock (hero, split classes, owe, math, cash flow, add button, tab bar — supersedes v5 as the approval target) + account-detail-v1 mock (the tap-through page: clean name, WHAT'S-INSIDE by type with readable security names, realized card, activity, read-only footer).</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>mockups/networth-v6-hifi-fullscreen-2026-07-19.html · mockups/account-detail-v1-hifi-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>MOCKS READY — v6 + account-detail await your approval</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
APPROVED + BUILT: NW class split, Mixed-holdings detail, WHAT'S-INSIDE, daily net-worth snapshots; FINAL mocks labeled
Split: accountClassBreakdown (slices sum EXACTLY to broker total; small
remainder folds to largest slice, material goes to mixed; manual accounts
never split) drives assetAllocation + per-class portion rows with plain
'in this account' words. Detail: multi-type accounts read 'Mixed holdings';
WHAT'S INSIDE · BY TYPE with readable names, class dots, cash row, options.
Daily snapshots: captureDailyNw (one point/day, DAILY_KEEP retention) +
trendPoints(monthly, daily) → graph within days. FINAL mocks:
networth-v7-hifi-FINAL + account-detail-v1-hifi-FINAL. 1239 green.
Workbook rows 15-16.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1043,6 +1043,86 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Net worth — graph with 1 month history?</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Can we not get 1 month history to show the graph?</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>No honest source exists for past values yet: the broker gives current balances only, and reconstructing history needs daily closing prices (the open price-provider decision). Drawing a line without them would be invented data.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED + BUILT: DAILY net-worth snapshots — one point per open day, bounded retention, trend draws within days. Full multi-year backfill (transactions × daily closes) lands with the price-provider decision.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>networth-v7 FINAL (legend note)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>BUILT — graph appears within days of Build 44</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Approvals — v6/account-detail/daily snapshots</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Go with daily snapshot change now. I approve account detail mockup — label it final. Revise NW mock with this change and label it final.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>ALL BUILT + pinned: class split (slices sum exactly; manual accounts whole; W8 walk proves the split), Mixed-holdings line, WHAT'S-INSIDE-BY-TYPE with readable names + cash row + option rows, daily snapshots wired Home→store→NW trend. FINAL mocks saved: networth-v7-hifi-FINAL + account-detail-v1-hifi-FINAL.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>networth-v7-hifi-FINAL-2026-07-19.html · account-detail-v1-hifi-FINAL-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>BUILT — 1239 tests green</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Invest v2 mock: winners/laggards capped at purchase date (founder finding row 17) — awaiting approval
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1123,6 +1123,46 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Invest — winners/laggards window</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>With 1Y selected, winners/laggards use one year even when the purchase is younger — LCTX shows as a winner over 1 year but is a loser since purchase. Show period or purchase date, whichever is shorter?</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed: rows show the SECURITY's period return; users read them as THEIR return. Opposite verdicts possible (the LCTX case).</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>RECOMMENDED + MOCKED (awaiting approval): window caps at purchase date; capped rows labeled "since you bought · Mar 3"; market comparison capped to the SAME dates; headline renamed YOUR RETURN, follows the same rule, notes when holdings are capped; dollar figures = value − cost (agrees with realized/unrealized math). Engine ready: lots carry purchase dates; BUY ledger rows fill gaps.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>mockups/invest-v2-hifi-capped-returns-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>MOCK AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Look-ahead hi-fi mock (as built, both states) + 3-item wireframe delta flagged for founder decision (workbook row 18)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1163,6 +1163,46 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Look ahead — objective + mock</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>What is the objective of Look ahead and what does the screen look like?</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Objective: answer "if I put away more each month, what does it buy me?" with the user's real numbers — the delta in dollars by retirement age + the will-it-last odds — labeled estimate, changing nothing. Sibling of Look back (past, facts).</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Hi-fi mock drawn from the BUILT screen (both states). HONESTY FLAG — 3 approved-wireframe items the built screen lacks: growth-rate pick (5/6/7%), bad-to-good markets range, "Use this plan" adopt button (adoption lives in Plan tab as built). FOUNDER DECIDES: add to match wireframe, or bless the simpler build.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>mockups/lookahead-v1-hifi-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>MOCK DELIVERED — 3-item wireframe delta awaits your call</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Build 44 (if changes)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Look-ahead gate diagnoses the TRUE blocker (build-43 finding, workbook row 19)
The dial renders only when the payoff can compute. The empty state names
what's actually missing and routes there: no accounts → connect chooser;
accounts in but plan basics missing (the founder's device case, now a named
pin) → 'Answer the plan questions' → Plan tab; unearmarked accounts → their
pages. v2 mock supersedes v1. 1242 green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,46 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Look ahead — confusing empty state</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Screen shows "If you add more each month $500" AND "Add your accounts and plan basics first… no guessed numbers"; Add accounts goes to Net worth. So confusing.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Three defects: (1) the dial rendered even when nothing could be computed — a dead control; (2) the gate lumped "accounts and plan basics" and blamed accounts — but you HAVE accounts; the true blocker was plan basics (your age/retirement inputs); (3) the button's words didn't match its destination.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>FIXED + pinned: the dial renders only when the payoff can; the gate diagnoses the TRUE blocker — no accounts → "Connect or add an account" (opens the connect chooser); accounts in but plan missing (YOUR case) → "Answer the plan questions" (opens Plan); accounts unearmarked → "Open your accounts". Your exact device state is a named test.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>mockups/lookahead-v2-hifi-fixed-empty-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Look-ahead v3 mock (inline age/retire-at sliders → canonical fields; info dots on delta + nest egg) + detailed design v1.2 with changelog — awaiting founder approval
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1243,6 +1243,46 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Look ahead — inline inputs redesign</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Screen should ask age (slider, saved) and retire-at (slider) right there; projected nest egg computed as they enter. Reduce friction, no duplicate fields, update detailed design doc. Info dots on nest egg and on the $243,000 number explaining the estimate.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Direction taken as PM/UX. Engineering note: native slider components add a native dependency, so the sliders are a pure-JavaScript control — same feel, no build risk.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>MOCK v3 delivered: dial + ABOUT YOU slider card (age 25–80, retire-at 50–75, "✓ Saved — Home, Plan and this screen all use these same answers"), payoff card with info dots on the delta AND on Projected nest egg (same plain-English how-we-calculate text), live recompute. Fields canonical: age→birthYear, retire-at→retirementAssumptions.retireAge (the Plan hub's own field). Detailed design bumped to v1.2 (v1.1 kept) with changelog tab. Plan-basics empty state dissolves — the sliders ARE the questions.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>mockups/lookahead-v3-hifi-inline-inputs-2026-07-19.html · FCC-core-detailed-design-v1.2-2026-07-19.xlsx</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>MOCK + DESIGN v1.2 AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cash flow first-day mock: inline 2-question setup replaces the $0 wall (workbook row 21) — awaiting approval
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1283,6 +1283,46 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow — $0 wall</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Shows $0 for all, with no opportunity to add income and spending to start with.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed in code: the working-lens hero renders In/Out/Surplus + pace bar with zeros when income/spending were never captured — no gate, no inline door. Same disease as What-if: the screen needs data it never asks for.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>MOCK for approval (your reduce-friction pattern): first day replaces the zero-hero with TWO inline questions — take-home per month + typical monthly outgo — saved to the SAME canonical plan fields Home/Budget/Plan read (no duplicates); ＋Expense stays for real entries; no zeros anywhere until answered. The real screen appears the moment both are in.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>mockups/cashflow-v1-hifi-inline-setup-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>MOCK AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Founder copy for the nest-egg info dot (near-verbatim, pinned) + professional table alignment on Invest rows (rows 22-23)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,86 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Look ahead — info dot copy</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Info dot explanation of nest egg and estimate not clear — use the simpler supplied wording.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Your wording adopted near-verbatim (the example figure generalized to "the amount shown" since the dot sits beside changing numbers). Pinned phrase-by-phrase.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — your copy is live</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Invest — row alignment</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Winners/laggards + investment details layout not professional: ▲/▼ wrapping to two lines; numbers not aligned (pushed right on long text, floating after short text).</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Arrow column too narrow for "⚠ Laggard:" (wrapped); dollar column had no fixed width or right alignment, so it followed the text instead of sitting in a column.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Proper table columns: arrow column widened + never wraps (one line enforced); dollar and percent columns right-aligned with fixed minimum widths and tabular figures — every row lines up regardless of name length. Applied to winners/laggards AND the holdings list.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>matches invest-v3 FINAL (its rows were already drawn aligned)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Invest 'all three' BUILT: dividends disclosure + mix-matched benchmark label + portfolio weights (row 24); invest-v4 FINAL mock
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1403,6 +1403,46 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Invest — investor-review items ("all three")</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Approved all three: dividends disclosure, benchmark relabel, portfolio weights.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>From the 45-year-old-investor review: returns are price-only (dividends excluded); "vs the stock market" mislabels the mix-matched blend; no weights column.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>BUILT + pinned: (1) "price changes only — dividends not included" line + ⓘ Price-returns glossary (total-return tracking noted as arriving with the price provider); (2) "vs the market, matched to your mix" + ⓘ benchmark; (3) gray weight % beside every holding and bond/alt account row, right-aligned column. FINAL mock updated to v4.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>mockups/invest-v4-hifi-FINAL-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>BUILT — 1244 green</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Invest v5 mock: statement-grade rows (arrow inside the right-aligned figure, fixed columns, subs under names) + one-line footnote with a single explain-everything dot — awaiting approval (row 25)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1443,6 +1443,46 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Invest — rows still not professional + footnote pile</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Winners/laggards and holdings still not aligned (arrow/name/number stacking, numbers not in one column); "since purchase — marked below / price changes only / prices updated" stack not easy to understand.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>v4 kept a separate arrow column and let notes share the number line — mixed one- and two-line rows with ragged figures. The three hero footnotes read as a jargon pile.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>MOCK v5 (awaiting approval): statement-grade rows — the arrow lives INSIDE the right-aligned figure ("▲ +$7,620 · +41%" as one unit, one x-position every row); holdings = fixed columns weight·value·return·›; sub-notes sit under the NAME only; the three footnotes collapse to ONE line "How these numbers work ⓘ · prices updated 2h ago" whose ⓘ explains purchase-capping, same-dates market matching, and the dividends exclusion in plain English.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>mockups/invest-v5-hifi-statement-rows-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>MOCK AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Invest v6 mock: winners/laggards as a true table (headers, split $/% columns) + holdings-list headers; info-dot copy in chat for approval (row 26)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1483,6 +1483,46 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Invest — make winners/laggards a real table</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Why not create a table for winners and laggards? And what is the info-dot text for "How these numbers work"?</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Agreed — a header row + split columns beats a combined figure; it is the brokerage-statement pattern.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>MOCK v6 (supersedes v5): true table — header HOLDING · CHANGE · RETURN, dollars and percents in separate right-aligned columns, arrow inside the CHANGE cell; the holdings list gets the same header (HOLDING · WEIGHT · VALUE · RETURN). Info-dot copy delivered in chat for approval: counted from purchase (yours, marked) + market same dates matched to your mix + prices only, dividends not included.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>mockups/invest-v6-hifi-table-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>MOCK + ⓘ COPY AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Invest v7 mock: header cells share the row-column widths; header placed under the first asset-class heading (row 27)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1523,6 +1523,46 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Invest — header alignment + placement</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Weight header not aligned with the weight column; place the header below Stocks/ETFs (the first asset class).</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>The header cells were not bound to the same fixed widths as the row cells; and the header sat above the class heading.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>MOCK v7: header cells share the exact row-column widths (aligned by construction); the column header now sits directly under the FIRST class heading, labeling the whole list once.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>mockups/invest-v7-hifi-table-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>MOCK AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v7 FINAL BUILT: winners/laggards as a true table (HOLDING·CHANGE·RETURN headers, split $/% right-aligned columns, arrow inside CHANGE, Leader/Laggard words not emoji) + holdings-list header under the first class (HOLDING·WEIGHT·VALUE·RETURN) + ONE footnote dot with the founder-approved howReturnsWork copy. invest-v7 FINAL mock labeled. 1244 green. Rows 25-27 closed.
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -1474,7 +1474,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>MOCK AWAITING APPROVAL</t>
+          <t>APPROVED + BUILT (v7 FINAL) — table headers, split $/% columns, one footnote dot (founder copy verbatim), pinned</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>MOCK + ⓘ COPY AWAITING APPROVAL</t>
+          <t>APPROVED + BUILT (v7 FINAL) — table headers, split $/% columns, one footnote dot (founder copy verbatim), pinned</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>MOCK AWAITING APPROVAL</t>
+          <t>APPROVED + BUILT (v7 FINAL) — table headers, split $/% columns, one footnote dot (founder copy verbatim), pinned</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Income pop-up mock (stable/variable, canonical fields) + keyboard class-fix accounting (rows 28-29; row 21 superseded)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>MOCK AWAITING APPROVAL</t>
+          <t>SUPERSEDED by row 28 (income becomes a pop-up); the spending question stays inline</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1558,6 +1558,86 @@
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Income capture — pop-up with stable/variable</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Instead of asking to enter income on Cash flow, make income a pop-up. Ask if income is stable or variable; design a way to capture both.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Supersedes the row-21 inline-questions mock (income part).</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>MOCK ready: Cash flow first day offers "Set up your income ›" opening a sheet — Q1 "How steady is it?" (Same every month ✓ / It varies). Steady → one take-home amount. Variable → typical month + tap-to-adjust 12-month grid (writes the EXISTING by-month income table Plan and taxes read — no duplicate fields). Reachable from every income edit point. Keyboard-safe sheet.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>mockups/income-popup-v1-hifi-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>MOCK READY — say yes to build, or mark it up</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard covers input screens (recurring)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Edit base salary — screen completely behind keyboard. Identified over and over, claimed fixed every time, still not fixed. Explain the technical difficulty.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>HONEST ANSWER: no remaining technical difficulty. History: the original third-party keyboard library was incompatible with our React Native version (logged 2026-06-25); a correct in-house fix (KeyboardAwareScreen/Sheet + the iOS scroll-inset) was then built — but applied screen-by-screen: only 11 of 31 input screens were converted, with NO guard. Each "fixed it" was true for that screen; the class was never closed. The base-salary editor was among the 20 unconverted.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>CLASS CLOSED TODAY: all 20 remaining input screens converted in one sweep (base-salary editor included), and keyboard_guard.test.ts permanently FAILS the build if any screen with a text input lacks keyboard handling — zero exceptions, no baseline. 1245 tests green.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>FIXED AS A CLASS + permanent guard</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Build 44</t>
         </is>

</xml_diff>

<commit_message>
Money IA redesign: research doc + ONE-surface four-tab mock (Cash flow·Income·Spending·Debts) — awaiting founder approval (row 30)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1643,6 +1643,46 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Money IA — Budget vs Cash flow duplication</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Budget screen (Activity/Budget/Debts) and Cash flow screen show the same information in different formats. Rethink: one screen, four tabs — income, expenses, debt, budget/cashflow. Research as principal product leader; best-in-class, simple, crisp.</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed in code: both screens compute the same month math (budgetVsActual, same income source) — true duplication. Industry research (Simplifi, Copilot, Monarch, YNAB, Rocket Money): winners MERGE plan-vs-actual into the cash-flow month view; none ship budget+cashflow as siblings.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>PROPOSAL (mock + research doc): ONE Money surface, four tabs — Cash flow (default; budget folded in: hero, pace, category plan, month bars), Income (sources + the approved steady/varies pop-up + received-this-month), Spending (activity + BIG-TICKET RADAR + categories vs plan + import), Debts (balances, pay-first, log payment, progress). Budget screen retires; same engines, no new fields; retiree lens keeps paycheck-first hero.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>mockups/money-v1-hifi-4tabs-2026-07-19.html · docs/FCC-core-55-70/money-ia-redesign-v1-2026-07-19.md</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>MOCK + RESEARCH AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cash flow surface v2 mock: name recommendation (Cash flow · This month tab), all 4 first-open states, all 6 linked screens, Teller-ready source chips + dedupe seams (row 31)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1683,6 +1683,46 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow surface — name, first-open, linked screens</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Don't call it Money (money is everything). Show first-open states and all linked screens (expense, edit plan, set up income, transactions search, import statement, log payment). Remember Teller will import transactions directly.</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>NAME RECOMMENDED: "Cash flow" (already the tab-bar name — zero ripple; covers in AND out; "Budget" would misname income/debt tabs); first tab renamed "This month" to kill the redundancy. MOCK v2 delivers: all 4 first-open states (no zeros anywhere — setup doors instead, bank-connect doors marked SOON) + all 6 linked screens (approved ＋Expense grid; Edit-plan sheet with live In−Plan−Debt=Left-over math; the approved income pop-up in place; transactions+search with SOURCE CHIPS bank/imported/by-hand — the Teller dedupe seam; statement import with big-ticket flag + no-duplicates gate + becomes-automatic note; log-a-payment with the one-entry no-double-count promise).</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>mockups/cashflow-v2-hifi-firstopen-and-links-2026-07-19.html</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>MOCK AWAITING APPROVAL (name pick + screens)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cash flow surface: month switcher (past=frozen actuals, future=labeled plan) added to the v2 mock, section C (row 32)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1723,6 +1723,46 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow surface — prior/future months</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Where to find cashflow, income, spending, and debts for prior months or future?</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>The four-tab mock lacked a time control.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>ADDED to the v2 mock (section C): one ‹ month › switcher under the title steers ALL FOUR tabs. Past months = frozen actuals (In received / Out spent / surplus / vs-plan verdict; that month's transactions, income, payments) from the existing month snapshots. Future months = the plan, labeled "planned — an estimate" (expected income incl. by-month variable table; usual spending + dated big bills like Nov property tax; scheduled debt payments) from the existing dated grid. Month bars stay as quick-jump. No new engines.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>mockups/cashflow-v2-hifi-firstopen-and-links-2026-07-19.html (section C)</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>IN THE MOCK AWAITING APPROVAL</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Build 44</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Screen review index: every screen, its mock status, and its Build-43 path (new workbook tab)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Build 43 feedback" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Screen review index" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1766,4 +1767,1166 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Mock-up (mockups/ folder)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>How to reach it in Build 43</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>What changes in Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>✅ FINAL — mock approved</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>home-investments-card-build44… + home-v2-hifi + approved-wireframes-home-networth</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Tab bar → Home</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Investments ⓘ · $-change+date always · net-worth line · splash fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Net worth</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>✅ FINAL — mock approved</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>networth-v7-hifi-FINAL (v2–v6 superseded)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Tab bar → Net worth</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Class split w/ portions · expand/collapse · clean names · daily-graph · as-of date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Invest (main)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>✅ FINAL — mock approved</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>invest-v7-hifi-table-FINAL (v1–v6 superseded)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Tab bar → Invest</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>YOUR RETURN hero · capped returns · true tables w/ headers · weights · one ⓘ footnote</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Account detail</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>✅ FINAL — mock approved</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>account-detail-v1-hifi-FINAL</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Net worth → tap a class open → tap an account</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-holdings line · WHAT'S INSIDE by type · readable CD names · activity arrives (sync self-heal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>What if I save more (Look ahead)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>✅ FINAL — mock approved</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>lookahead-v3-hifi-inline-inputs-FINAL (v1–v2 superseded)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Invest → "LOOK AHEAD" card</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Inline age/retire-at sliders (saved) · ⓘ on delta + nest egg (your wording) · smart empty states</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow — NEW 4-tab surface (This month · Income · Spending · Debts)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>🟨 AWAITING YOUR APPROVAL</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>cashflow-v2-hifi-firstopen-and-links (sections A+B+C) — supersedes money-v1 + cashflow-v1</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Compare against: Tab bar → Cash flow AND Menu → Budget (the two screens it merges)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>THE consolidation: name pick + approval pending; month switcher; Teller-ready doors</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>— Income pop-up (steady/varies)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>✅ direction approved — rides the Cash-flow build</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>income-popup-v1-hifi</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>n/a (new)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Lives in the Income tab; writes canonical fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Budget screen (Activity/Budget/Debts/Import)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>🔴 RETIRES (absorbed) on Cash-flow approval</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>n/a — its jobs move into the new surface</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Menu (☰) → Budget &amp; activity</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Retires; Activity→Spending, Budget→This month plan, Debts→Debts tab, Import→Spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Income manager family (income-manager · monthly-income · income-detail · paycheck-months)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>🟨 folds under the Income tab (pop-up + by-month grid stay as its editors)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>income-popup-v1-hifi</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Menu → Income / Sharpen → income; retiree: Cash flow → "See July's paycheck"</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Reached from Income tab; keyboard fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Job safety</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>✅ FINAL (approved rebuild — already IN Build 43)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>jobsafety-rebuild-approved-2026-07-17</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Plan → Job safety (working lens)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>None further</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>＋ Expense sheet</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved 7/16 — already IN Build 43</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>(drawn again in cashflow-v2 §B, unchanged)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow → ＋ Expense</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>None further</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Connect a brokerage (SnapTrade flow)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved design — IN Build 43 (you used it)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>n/a (built per approved design v2 §2)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Net worth → ＋ Add or connect → Link it</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>History self-heal · read-only consent line</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Plan hub</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>(approved wireframes only)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Tab bar → Plan</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Global only (keyboard, glossary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Retirement cockpit</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Plan → the cockpit card</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Will my money last</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Home → the odds strip → full picture</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Social Security timing</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Plan → Social Security timing</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Roth</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Plan → Roth</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Required withdrawals (RMD)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Plan → Required withdrawals</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Stress test</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Plan → stress test (via Insurance card)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Tax organizer</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Menu → Tax organizer</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Goals · Multi-goal</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Plan → Goals / Menu</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Month detail</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Cash flow → tap a month bar</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Reached via the new month switcher too</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Bill calendar</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Menu → Bill calendar</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Feeds the future-month view</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Look back</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>(approved wireframe)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Invest → "LOOK BACK" card</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Holding detail (stock/fund)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>(wireframe; realized-P/L card already in 43)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Invest → tap a holding</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Capped-return label consistency</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Bonds editor</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Net worth → a bond → edit / Invest → bond row</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Other investments (alternatives editor)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Invest → an alternative → edit</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Add account (by hand)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Net worth → ＋ → Add by hand</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Import holdings (CSV)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Net worth → ＋ → Import from a file</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Options class correctly (OCC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Settings (incl. connected accounts)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Home → gear</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Sharpen</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Menu → Sharpen your plan</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Income door points at the new pop-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Insights</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Home → an insight card / Menu</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Worth a look</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>(approved wireframe)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Home → the ◆ Worth-a-look card (when flagged)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Contribution room (401k)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Home → the 401(k)-room item</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Idle cash</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Home → the idle-cash item</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Education · Tips · Rewards · Savings (legacy)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Menu → Tools &amp; check-ups</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Review: candidates to retire post-launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Credit · Insurance · Estate</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Menu → Tools &amp; check-ups</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Insurance stress-link · Recovery modal</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>via Insurance / recovery prompts</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Onboarding / first-run</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved — IN Build 43</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>(approved wireframes, Home tab sheet)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Fresh install or Settings → restart setup</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>None further</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Auth (sign in)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>⬜ SAME as Build 43 — review on device</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Sign out → sign-in screen</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Global only</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
BUILD-44 feedback fixed: receipt total-vs-cash + variable-income year frames (rows 33-34)
Receipt (both parsers): payment-mechanics lines never count; last explicit
total wins; subtotal → largest-safe fallbacks. Founder's exact receipt
pinned (TOTAL 56.47 beats CASH 100.00) + 3 edge cases; pins pierce the ui
project's global receiptScan mock via requireActual.

Income sheet: 'Which 12 months are you entering?' — Calendar year N or Next
12 months; chips + editors carry real month+year labels incl. across the
New-Year boundary; both frames write the same canonical calendar slots
(salaryByMonth is a repeating yearly pattern — verified in the engine).
1256 green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1761,6 +1761,86 @@
       <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Build 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>BUILD 44 · Receipt scan — captured cash paid, not the total</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>When I scan a receipt it captured cash paid versus balance.</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Both parsers (on-device + the Vision fallback) kept the LARGEST number on the receipt — and the CASH TENDERED line ($100 handed over) is usually bigger than the bill ($56.47).</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>FIXED in both parsers, human reading rules: amounts on payment-mechanics lines (cash/tendered/change/card/auth…) are NEVER candidates; the LAST explicit TOTAL/AMOUNT-DUE/BALANCE-DUE line wins (grand total beats a mid-receipt total); subtotal then largest non-payment amount are the fallbacks. Pinned with your exact scenario + 3 edge receipts.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>n/a (engine)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 45</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>BUILD 44 · Variable income — no year, ambiguous 12 months</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Months show no year; Jan–Dec 2026 not feasible — it reads as Aug 2026–Jul 2027. Let the person choose calendar year or 12 months from today, smartly.</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>The by-month table is calendar-indexed (Jan→Dec, a pattern repeating each year) but the chips carried no year and no frame choice — ambiguous exactly as you described.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>FIXED per your design: a new question "Which 12 months are you entering?" with two chips — Calendar year 2026 (Jan ’26 … Dec ’26) or Next 12 months (Aug ’26 … Jul ’27, real years across the boundary). Both write the SAME canonical slots; every chip and editor now carries month + year; honest note "this yearly pattern repeats". Pinned incl. the year-boundary labels.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>final mock updated on your next approval pass</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 45</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B44 fix: table header cells share ONE 10.5pt header type (column styles = width/alignment only), single-line — RETURN can't wrap (row 35)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1839,6 +1839,46 @@
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>BUILD 44 · Invest table headers — mixed sizes, RETURN wraps</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Winners &amp; laggards: font sizes of HOLDING, CHANGE and RETURN differ; the N of RETURN wraps to the next line.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Style-ordering bug: header cells combined header typography with the COLUMN styles, column styles last — so the data cells' 14pt/13pt sizes overrode the header's 10.5pt, and 13pt "RETURN" no longer fit its 62px column.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>FIXED in both tables: column styles now supply width/alignment ONLY (listed first), header typography wins (listed last), and every header cell is locked to one line. Pinned: all header cells assert the SAME 10.5pt + single-line.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 45</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Build 45</t>
         </is>

</xml_diff>

<commit_message>
B44 findings 3-6 fixed: alt-row overlap (pinned w/ founder's QQQ row), investments-list chip/size cleanup, holding-detail cents precision (maskedMoney2), honest options About-box (no fake 'typical return' for contracts; 14pt fact rows). Row 40 logged: Spending-vs-mock conformance restyle underway. 1257 green.
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1879,6 +1879,206 @@
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>B44 · Alternatives row overlap</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>QQQ Dec 31 ’26 option row: "Value as of" overlaps with $1,408.</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>My earlier alignment change removed the flexible width from row names — long option labels stopped shrinking and collided with the chip and amount.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: the label shrinks (truncates) again; chip and amount keep their columns. Pinned with your exact row (QQQ $600 put · exp Dec 31 2026 at $1,408).</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 45</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>B44 · Investments list — mixed sizes + "44% Live" jam</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Your-investments table labels all different sizes; the weight column shows "44% Live".</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>The Live/Prices-old chip sat BETWEEN the weight and value columns, and the name rendered one size larger than the value.</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: the chip moved in next to the NAME (columns stay pure: name · weight · value · return · ›), and the name now matches the value size (14pt).</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 45</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>B44 · Holding detail — integers everywhere</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>All numbers are integer versus float.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Every money figure was rounded to whole dollars.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: money on the holding page is cents-precise (value, gain, average cost, lots, realized, dividends) via a new masked cents formatter; percentages and the ~estimated tax (a labeled estimate) unchanged. Pins updated to the cents truth.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 45</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>B44 · Options About-this-holding box</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Type "options" bold/different size; "Typical yearly return for this type ~5.0% estimate from history" — not the design I agreed to.</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>The About box is the APPROVED design for gold/crypto (the wireframe shows "Typical yearly return ~8.2% · estimate from history") — but options were never contemplated there, and a typical yearly return for an option CONTRACT is not an honest number.</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: for options the line is replaced with the truth ("Options are contracts — no typical yearly return exists; value moves with the underlying, time and volatility"); fact rows now one size (14pt). Classic alternatives keep the approved line.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>per approved wireframe (alternatives frame)</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 45</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>B44 · Spending tab ≠ the approved mock</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Spending screen — this [the mock] is the mock-up I agreed to.</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>The Spending tab embeds the old Activity body for its proven money logic — correct engine, but it carries the OLD look (strip, filters), not the approved §B layout (big-ticket radar, clean day-grouped list with source chips, categories vs plan).</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>IN PROGRESS: restyling the Spending tab to the approved mock exactly (the radar is already in; the list presentation and source chips come next). The approved mock is the spec — no re-approval needed, this is conformance work.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>mockups/final/cashflow-4tabs-FINAL-2026-07-19.html §A/§B</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — conformance restyle underway</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Build 45</t>
         </is>

</xml_diff>

<commit_message>
Teller access verified gated (no public signup; /signup 404) — founder email path + cert/relay integration plan logged (row 41)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2081,6 +2081,46 @@
       <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Build 45</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Teller — signup access</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Cannot find how to sign up for Teller.</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED 2026-07-19: teller.io currently exposes NO public signup — the homepage has only "Sign in" (email/password), teller.io/signup returns 404, and the docs assume an existing account. Access appears gated: their free developer tier (100 live connections) is still advertised, so they DO onboard — by request.</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>ACTION (founder): email hello@teller.io requesting a developer account (draft provided in chat). AFTER access: signup auto-generates teller.zip (client certificate + private key = SECRETS → same Firebase-relay pattern as SnapTrade, never in the app) + an application id (non-secret) from Dashboard → Application Settings. Sandbox is free/unlimited; development tier = 100 free live connections. FALLBACK if no reply in ~1 week: revisit bank-connect research (SimpleFIN Bridge is the self-serve indie option).</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>docs/FCC-core-55-70/bank-connect-research-2026-07-18.md</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>WAITING ON TELLER ACCESS (founder email)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>post-45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Launch sign-off + index: onboarding flow expanded into its 5 distinct screens (45 rows total)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -2135,7 +2135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3286,6 +3286,156 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>First run · Step 1 — value intro</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved flow — IN the build</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>(approved first-run flow map, Home tab sheet)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Fresh install → the first screen (what MoneyKeel can do + the read-only promise)</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Approved first-run flow; skippable</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>First run · Step 2 — the two questions</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved flow — IN the build</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>(approved first-run flow map, Home tab sheet)</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>"What did you come for?" (pick all) + "Where are you these days?" (working / retired) — after the intro; also Settings → Your setup</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Sets the lens + tab order; answers only order suggestions</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>First run · retiree fast-path — Monthly income</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved flow — IN the build</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>(approved first-run flow map, Home tab sheet)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Answer "retired" + "a retirement paycheck" in step 2 → the 2-number Social Security / pension screen, no bank login</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>The retiree快 path; feeds the paycheck hero</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Full setup questionnaire (multi-step)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved flow — IN the build</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>(approved first-run flow map, Home tab sheet)</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Settings → restart setup (or Sharpen → full setup) — walk every step: status, income, salary, spending, retirement…</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>The deep wizard; every step skippable with sensible defaults</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Home · first-run empty state (the doors)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>✅ approved flow — IN the build</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>(approved first-run flow map, Home tab sheet)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Fresh account before any data — Home shows "Let's get your real numbers in" with Connect / Add by hand doors</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>No fake zeros; the two doors + what-you'll-see preview</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sentry B-L2 verify (founder) + optional read-token (mine) saved as tracked to-dos (rows 42-43)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2121,6 +2121,86 @@
       <c r="H42" s="2" t="inlineStr">
         <is>
           <t>post-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>LAUNCH GATE · Sentry B-L2 verification (YOUR to-do)</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Fire the test event and confirm it lands: phone → Settings → Legal &amp; Support → "Send a diagnostic report" → sentry.io (org finwise-35, project react-native) shows the event within ~1 min.</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>The June launch checklist's last B-L2 step (🧑) — never completed through builds 34–45; re-surfaced 2026-07-21.</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Open item until you confirm. Closes B-L2 exactly as written in June.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>docs/finwise-sentry-setup.md §6</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — after your screen walk</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>launch gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>OPTIONAL · Sentry read token (MY to-do once you provide)</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Create a read-only token (sentry.io → Auth Tokens → org:read, project:read, event:read) → paste into a Desktop file I create → I store it in the gitignored .env, delete the file, and take over crash monitoring for beta.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Gives me direct error access so triage is mine during beta.</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>On your word — 3 minutes when convenient.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>OPEN — optional, when convenient</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>pre-beta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B45 CRITICAL: entry redirected to the OLD onboarding (pre-June leftover) — now lands on the auth gate, guard routes to the approved first-run (row 44)
app/index.tsx targeted /onboarding with a comment from the account-created-
mid-flow era; superseded twice (June auth-first, B42 light first-run). The
guard was right all along but treats /onboarding as legal (the by-hand
door), so nothing bounced the stale entry. Pins: the entry file can never
target /onboarding; the guard's auth→first-run→home routes asserted.
1260 green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2201,6 +2201,46 @@
       <c r="H44" s="2" t="inlineStr">
         <is>
           <t>pre-beta</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>B45 · Fresh install shows the OLD onboarding first</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Build 45 — first screen was old onboarding; skipping landed at MoneyKeel [the auth/brand screen].</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT RESULT: the app's ENTRY file still hard-redirected cold starts to /onboarding (the deep questionnaire), with a comment from the pre-June architecture ("account created mid-flow"). That flow was superseded twice (June: auth-first; Build 42: the approved light first-run) — the route GUARD is correct, but it deliberately treats /onboarding as a legal place to be (the by-hand door), so the stale entry redirect was never bounced. The guard's tests pass because the guard is right; nobody pinned the ENTRY file.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: the entry now lands on the auth gate and the guard does all routing (unauthenticated → sign in; new user → the approved first-run; returning user → Home). Two pins: the entry file can never target /onboarding again, and the guard's three routes are asserted. The deep questionnaire stays reachable ONLY by choice (Home's set-up-by-hand door, Settings → restart setup).</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 46</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Build 46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
B45 founder findings 46-50 fixed: wordmark = the logo ART everywhere, honest 'Securing' on sign-in envelope build, slider stale-closure touch bug, honest NW span label, single-security import naming heal
Rows 45-50 in the feedback workbook with verified root causes; plain-English
root-cause file docs/FCC-core-55-70/build45-feedback-root-causes-2026-07-24.md;
mock mockups/brand-wordmark-v1-2026-07-24.html; real-touch-path PlanSlider
tests; 1270 green, tsc clean, ui-test gate ok.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
+++ b/docs/FCC-core-55-70/build43-feedback-v1-2026-07-19.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2239,6 +2239,246 @@
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Build 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>B45 · Launch screen still black after the fix</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Latest build still shows MoneyKeel in black at launch.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED IN THE REAL ARTIFACT: I downloaded the exact Build-45 app file from the build server and looked inside — the approved colored splash IS baked in (full-size image, light and dark slots, white background). The black at launch on the device is the iPhone's launch-screen cache: iOS keeps serving the snapshot it took back when Build 43 shipped broken. Deleting the app alone is often not enough; the phone must restart too.</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>No code change needed (verified in the artifact). Clear steps: delete app -&gt; restart iPhone -&gt; reinstall. NOTE: most of what was called "black MoneyKeel" turned out to be row 46 — the sign-in screen — which reinstalls can never fix.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>VERIFIED — device cache, not the build</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>B45 · The MoneyKeel name matches the designed logo NOWHERE</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Sign-in screen shows the name in black; the rest of the app shows it in flat green; neither matches the designed logo.</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>The name was TYPED as text on every surface — sign-in typed it in near-black, the top bar typed it in flat green. Typed text can never match the designed logo: the logo is two-tone ("Money" teal, "Keel" navy) in its own typeface. The screens were each styled locally instead of using the logo art.</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: no screen types the name anymore. The actual wordmark art (cut from the approved logo file) now renders on sign-in, the welcome screen, and the top bar of every screen — one shared asset, pixel-true to the logo. Mock: mockups/brand-wordmark-v1-2026-07-24.html (built to match; flag if you want it different).</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>mockups/brand-wordmark-v1-2026-07-24.html</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 46</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Build 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>B45 · Sign-in: Welcome shows ~30 s, then the recovery code interrupts</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Welcome screen appears ~30 seconds, disappears, recovery code appears, then Welcome again.</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Your test account is HALF-DELETED: its data was removed from the database but its LOGIN still exists (that is also why the email says "already exists"). Signing into it makes the app treat it as an account that needs its encryption set up: it silently runs the deliberately-slow key-securing math (~30 s, security feature) with NO feedback on the sign-in path — the signup path already had an honest "Securing…" spinner, sign-in never got it. When the math finished, the code popped up over Welcome; returning to Welcome after is correct (the account has no data, so setup must run).</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: sign-in now shows the recovery-code sheet IMMEDIATELY with the honest "Securing your account…" spinner — same approved sheet, honest timing. YOUR STEP for clean testing: Firebase console -&gt; Authentication -&gt; Users -&gt; delete blah1@gmail.com; then the email is truly fresh and none of this path runs.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 46 · founder step open</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Build 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>B45 · What-if slider jumps to max on touch</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>The moment you touch the slider it goes to max — you cannot slide it.</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>The touch handler is created ONCE when the screen first draws and permanently remembered the track width from that instant — a 1-pixel placeholder, measured before the real width arrived. Every later touch divided by 1 px, computed a huge value, and clamped to the maximum. Our screen tests drive the slider through its accessibility path (which reads live values), so this touch-only bug passed every test — a class of bug only a real finger finds.</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: the handler now reads the CURRENT width and values on every touch (and a parent scroll can no longer steal the drag mid-gesture). New tests drive the REAL touch path with real coordinates — middle of track must select the middle value.</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 46</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Build 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>B45 · Net worth says "up $0 this year"</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Top of Net worth: Your net worth $169,530, up $0 this year.</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Two dishonesty bugs in one line. (1) The label lied about the span: "this year" implies a January baseline, but your history only started ~5 days ago, so it was really comparing to last week. (2) Your imported holdings have no live price feed yet (price provider still to be chosen), so the value genuinely had not moved — and an unchanged value was worded as "up $0".</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>FIXED: the label now tells the truth about the span — "this year" ONLY when the baseline really is January; a young history says "since Jul 19"; an unchanged value says "no change since Jul 19", never "up $0". Pinned for both cases.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 46</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Build 46</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>B45 · "E*TRADE Imported holdings" vs "E*TRADE LCTX"</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Under Stock/ETF one row says E*TRADE imported holding; the rest name the security (E*TRADE VMFXX).</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>The LCTX account was created by an OLDER import that used the generic default name "Imported holdings"; newer single-security imports are named by their ticker. Old data kept its old label — the naming rule changed but existing accounts were never healed.</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>FIXED in the one shared naming helper (every screen inherits): a generically-labeled account holding exactly ONE security now wears that security's name -&gt; "E*TRADE LCTX". Accounts with several holdings keep the honest generic name. Pinned.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>FIXED — rides Build 46</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>Build 46</t>
         </is>

</xml_diff>